<commit_message>
xd12 fault 관련 bit_mask define 추가, trim condition 적용
</commit_message>
<xml_diff>
--- a/XD_JIG/XD04/XD04_PWM_Rev_0/Docs/GT/XD_PWM_TEST_250320.xlsx
+++ b/XD_JIG/XD04/XD04_PWM_Rev_0/Docs/GT/XD_PWM_TEST_250320.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\Jig\XD_JIG\XD12\XD12_PWM_Rev\Docs\GT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\Jig\XD_JIG\XD04\XD04_PWM_Rev_0\Docs\GT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09BB1CE9-DC65-4026-8DBB-2EC28ED21824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49DBCD40-5D6A-41D7-8BC0-70116F186E2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="4095" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test_Plan" sheetId="2" r:id="rId1"/>

</xml_diff>